<commit_message>
Set supply target to 171.4 million users
</commit_message>
<xml_diff>
--- a/public/reports/personal-ai-compute-report-card.xlsx
+++ b/public/reports/personal-ai-compute-report-card.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rba501706d1884829"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R09737a5f1e3549bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R18d99d0205a84707"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R2cd2b82930ec4152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="Rc90da92a79de4c76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R4ac21b77e2934730"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3c2fbbc51d5e42b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Compute Report Card" sheetId="2" r:id="R90e4df5f120c4592"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quarterly Model" sheetId="3" r:id="R6317b6c2ae934b35"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="4" r:id="R6025b029246641bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Observations" sheetId="5" r:id="R7511e55f45c34d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="Rc60d5a6806284a58"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -470,7 +470,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc10e600d03eb4c4f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1ab68e3938d24ad3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -920,7 +920,7 @@
     <x:row r="6">
       <x:c r="A6" s="54" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37598995605326785</x:v>
+        <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="D6" s="55" t="n">
         <x:f>'Quarterly Model'!E16</x:f>
@@ -934,7 +934,7 @@
       </x:c>
       <x:c r="J6" s="57" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46631.98192288111</x:v>
+        <x:v>46632.108708204854</x:v>
       </x:c>
       <x:c r="M6" s="53" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
@@ -1014,11 +1014,11 @@
       </x:c>
       <x:c r="C14" s="29" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37598995605326785</x:v>
+        <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="D14" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46631.98192288111</x:v>
+        <x:v>46632.108708204854</x:v>
       </x:c>
       <x:c r="E14" s="17" t="str">
         <x:v>Waiting</x:v>
@@ -1077,7 +1077,7 @@
       </x:c>
       <x:c r="B20" s="19" t="n">
         <x:f>'Quarterly Model'!J6</x:f>
-        <x:v>0.00682986953450553</x:v>
+        <x:v>0.00682782226716592</x:v>
       </x:c>
       <x:c r="C20" s="19" t="n">
         <x:f>1</x:f>
@@ -1091,7 +1091,7 @@
       </x:c>
       <x:c r="B21" s="19" t="n">
         <x:f>'Quarterly Model'!J7</x:f>
-        <x:v>0.013212410193757892</x:v>
+        <x:v>0.01320844974682248</x:v>
       </x:c>
       <x:c r="C21" s="19" t="n">
         <x:f>1</x:f>
@@ -1105,7 +1105,7 @@
       </x:c>
       <x:c r="B22" s="19" t="n">
         <x:f>'Quarterly Model'!J8</x:f>
-        <x:v>0.020077810262916846</x:v>
+        <x:v>0.020071791898291506</x:v>
       </x:c>
       <x:c r="C22" s="19" t="n">
         <x:f>1</x:f>
@@ -1119,7 +1119,7 @@
       </x:c>
       <x:c r="B23" s="19" t="n">
         <x:f>'Quarterly Model'!J9</x:f>
-        <x:v>0.028148718558294105</x:v>
+        <x:v>0.02814028092242638</x:v>
       </x:c>
       <x:c r="C23" s="19" t="n">
         <x:f>1</x:f>
@@ -1133,7 +1133,7 @@
       </x:c>
       <x:c r="B24" s="19" t="n">
         <x:f>'Quarterly Model'!J10</x:f>
-        <x:v>0.0375667289867675</x:v>
+        <x:v>0.037555468283042195</x:v>
       </x:c>
       <x:c r="C24" s="19" t="n">
         <x:f>1</x:f>
@@ -1147,7 +1147,7 @@
       </x:c>
       <x:c r="B25" s="19" t="n">
         <x:f>'Quarterly Model'!J11</x:f>
-        <x:v>0.06635913961769906</x:v>
+        <x:v>0.06633924833009283</x:v>
       </x:c>
       <x:c r="C25" s="19" t="n">
         <x:f>1</x:f>
@@ -1161,7 +1161,7 @@
       </x:c>
       <x:c r="B26" s="19" t="n">
         <x:f>'Quarterly Model'!J12</x:f>
-        <x:v>0.08728779219871709</x:v>
+        <x:v>0.08726162750476324</x:v>
       </x:c>
       <x:c r="C26" s="19" t="n">
         <x:f>1</x:f>
@@ -1175,7 +1175,7 @@
       </x:c>
       <x:c r="B27" s="19" t="n">
         <x:f>'Quarterly Model'!J13</x:f>
-        <x:v>0.14710906322515388</x:v>
+        <x:v>0.14706496698305438</x:v>
       </x:c>
       <x:c r="C27" s="19" t="n">
         <x:f>1</x:f>
@@ -1189,7 +1189,7 @@
       </x:c>
       <x:c r="B28" s="19" t="n">
         <x:f>'Quarterly Model'!J14</x:f>
-        <x:v>0.17518649830077868</x:v>
+        <x:v>0.17513398579018094</x:v>
       </x:c>
       <x:c r="C28" s="19" t="n">
         <x:f>1</x:f>
@@ -1203,7 +1203,7 @@
       </x:c>
       <x:c r="B29" s="19" t="n">
         <x:f>'Quarterly Model'!J15</x:f>
-        <x:v>0.31204191629301636</x:v>
+        <x:v>0.31194838109141576</x:v>
       </x:c>
       <x:c r="C29" s="19" t="n">
         <x:f>1</x:f>
@@ -1217,7 +1217,7 @@
       </x:c>
       <x:c r="B30" s="19" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37598995605326785</x:v>
+        <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="C30" s="19" t="n">
         <x:f>1</x:f>
@@ -1231,7 +1231,7 @@
       </x:c>
       <x:c r="B31" s="19" t="n">
         <x:f>'Quarterly Model'!J17</x:f>
-        <x:v>0.503968053473009</x:v>
+        <x:v>0.5038169880198742</x:v>
       </x:c>
       <x:c r="C31" s="19" t="n">
         <x:f>1</x:f>
@@ -1245,7 +1245,7 @@
       </x:c>
       <x:c r="B32" s="19" t="n">
         <x:f>'Quarterly Model'!J18</x:f>
-        <x:v>0.6610888725937321</x:v>
+        <x:v>0.660890709854224</x:v>
       </x:c>
       <x:c r="C32" s="19" t="n">
         <x:f>1</x:f>
@@ -1259,7 +1259,7 @@
       </x:c>
       <x:c r="B33" s="19" t="n">
         <x:f>'Quarterly Model'!J19</x:f>
-        <x:v>0.8486854625531765</x:v>
+        <x:v>0.8484310673527545</x:v>
       </x:c>
       <x:c r="C33" s="19" t="n">
         <x:f>1</x:f>
@@ -1453,7 +1453,7 @@
     <x:mergeCell ref="B44:N44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R27a95f4f29ae4286"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd08d6a9077de4ce9"/>
 </x:worksheet>
 </file>
 
@@ -2246,114 +2246,114 @@
       </x:c>
       <x:c r="C6" s="45" t="n">
         <x:f>'Quarterly Model'!J6</x:f>
-        <x:v>0.00682986953450553</x:v>
+        <x:v>0.00682782226716592</x:v>
       </x:c>
       <x:c r="D6" s="45" t="str">
         <x:f>'Quarterly Model'!K6</x:f>
       </x:c>
       <x:c r="E6" s="45" t="n">
         <x:f>'Quarterly Model'!J7</x:f>
-        <x:v>0.013212410193757892</x:v>
+        <x:v>0.01320844974682248</x:v>
       </x:c>
       <x:c r="F6" s="45" t="n">
         <x:f>'Quarterly Model'!K7</x:f>
-        <x:v>0.006382540659252363</x:v>
+        <x:v>0.006380627479656559</x:v>
       </x:c>
       <x:c r="G6" s="45" t="n">
         <x:f>'Quarterly Model'!J8</x:f>
-        <x:v>0.020077810262916846</x:v>
+        <x:v>0.020071791898291506</x:v>
       </x:c>
       <x:c r="H6" s="45" t="n">
         <x:f>'Quarterly Model'!K8</x:f>
-        <x:v>0.0068654000691589535</x:v>
+        <x:v>0.006863342151469026</x:v>
       </x:c>
       <x:c r="I6" s="45" t="n">
         <x:f>'Quarterly Model'!J9</x:f>
-        <x:v>0.028148718558294105</x:v>
+        <x:v>0.02814028092242638</x:v>
       </x:c>
       <x:c r="J6" s="45" t="n">
         <x:f>'Quarterly Model'!K9</x:f>
-        <x:v>0.008070908295377259</x:v>
+        <x:v>0.008068489024134873</x:v>
       </x:c>
       <x:c r="K6" s="45" t="n">
         <x:f>'Quarterly Model'!J10</x:f>
-        <x:v>0.0375667289867675</x:v>
+        <x:v>0.037555468283042195</x:v>
       </x:c>
       <x:c r="L6" s="45" t="n">
         <x:f>'Quarterly Model'!K10</x:f>
-        <x:v>0.009418010428473397</x:v>
+        <x:v>0.009415187360615817</x:v>
       </x:c>
       <x:c r="M6" s="45" t="n">
         <x:f>'Quarterly Model'!J11</x:f>
-        <x:v>0.06635913961769906</x:v>
+        <x:v>0.06633924833009283</x:v>
       </x:c>
       <x:c r="N6" s="45" t="n">
         <x:f>'Quarterly Model'!K11</x:f>
-        <x:v>0.028792410630931554</x:v>
+        <x:v>0.028783780047050636</x:v>
       </x:c>
       <x:c r="O6" s="45" t="n">
         <x:f>'Quarterly Model'!J12</x:f>
-        <x:v>0.08728779219871709</x:v>
+        <x:v>0.08726162750476324</x:v>
       </x:c>
       <x:c r="P6" s="45" t="n">
         <x:f>'Quarterly Model'!K12</x:f>
-        <x:v>0.02092865258101803</x:v>
+        <x:v>0.020922379174670408</x:v>
       </x:c>
       <x:c r="Q6" s="45" t="n">
         <x:f>'Quarterly Model'!J13</x:f>
-        <x:v>0.14710906322515388</x:v>
+        <x:v>0.14706496698305438</x:v>
       </x:c>
       <x:c r="R6" s="45" t="n">
         <x:f>'Quarterly Model'!K13</x:f>
-        <x:v>0.05982127102643679</x:v>
+        <x:v>0.05980333947829114</x:v>
       </x:c>
       <x:c r="S6" s="45" t="n">
         <x:f>'Quarterly Model'!J14</x:f>
-        <x:v>0.17518649830077868</x:v>
+        <x:v>0.17513398579018094</x:v>
       </x:c>
       <x:c r="T6" s="45" t="n">
         <x:f>'Quarterly Model'!K14</x:f>
-        <x:v>0.028077435075624796</x:v>
+        <x:v>0.02806901880712656</x:v>
       </x:c>
       <x:c r="U6" s="45" t="n">
         <x:f>'Quarterly Model'!J15</x:f>
-        <x:v>0.31204191629301636</x:v>
+        <x:v>0.31194838109141576</x:v>
       </x:c>
       <x:c r="V6" s="45" t="n">
         <x:f>'Quarterly Model'!K15</x:f>
-        <x:v>0.1368554179922377</x:v>
+        <x:v>0.13681439530123482</x:v>
       </x:c>
       <x:c r="W6" s="45" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37598995605326785</x:v>
+        <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="X6" s="45" t="n">
         <x:f>'Quarterly Model'!K16</x:f>
-        <x:v>0.06394803976025148</x:v>
+        <x:v>0.06392887120475099</x:v>
       </x:c>
       <x:c r="Y6" s="33" t="n">
         <x:f>'Quarterly Model'!J17</x:f>
-        <x:v>0.503968053473009</x:v>
+        <x:v>0.5038169880198742</x:v>
       </x:c>
       <x:c r="Z6" s="33" t="n">
         <x:f>'Quarterly Model'!K17</x:f>
-        <x:v>0.12797809741974114</x:v>
+        <x:v>0.12793973572370743</x:v>
       </x:c>
       <x:c r="AA6" s="33" t="n">
         <x:f>'Quarterly Model'!J18</x:f>
-        <x:v>0.6610888725937321</x:v>
+        <x:v>0.660890709854224</x:v>
       </x:c>
       <x:c r="AB6" s="33" t="n">
         <x:f>'Quarterly Model'!K18</x:f>
-        <x:v>0.15712081912072307</x:v>
+        <x:v>0.15707372183434987</x:v>
       </x:c>
       <x:c r="AC6" s="33" t="n">
         <x:f>'Quarterly Model'!J19</x:f>
-        <x:v>0.8486854625531765</x:v>
+        <x:v>0.8484310673527545</x:v>
       </x:c>
       <x:c r="AD6" s="33" t="n">
         <x:f>'Quarterly Model'!K19</x:f>
-        <x:v>0.1875965899594444</x:v>
+        <x:v>0.18754035749853049</x:v>
       </x:c>
       <x:c r="AE6" s="33" t="n">
         <x:f>'Quarterly Model'!J20</x:f>
@@ -2361,7 +2361,7 @@
       </x:c>
       <x:c r="AF6" s="33" t="n">
         <x:f>'Quarterly Model'!K20</x:f>
-        <x:v>0.15131453744682355</x:v>
+        <x:v>0.15156893264724547</x:v>
       </x:c>
       <x:c r="AG6" s="33" t="n">
         <x:f>'Quarterly Model'!J21</x:f>
@@ -2405,7 +2405,7 @@
       </x:c>
       <x:c r="AQ6" s="29" t="n">
         <x:f>'Quarterly Model'!J16</x:f>
-        <x:v>0.37598995605326785</x:v>
+        <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="AR6" s="29" t="str">
         <x:f>'Quarterly Model'!L16</x:f>
@@ -2417,7 +2417,7 @@
       </x:c>
       <x:c r="AT6" s="20" t="n">
         <x:f>'Assumptions'!B32</x:f>
-        <x:v>46631.98192288111</x:v>
+        <x:v>46632.108708204854</x:v>
       </x:c>
       <x:c r="AU6" s="27" t="n">
         <x:f>'Assumptions'!B30</x:f>
@@ -2683,7 +2683,7 @@
       </x:c>
       <x:c r="J6" s="29" t="n">
         <x:f>MIN(1,I6/'Assumptions'!$B$9)</x:f>
-        <x:v>0.00682986953450553</x:v>
+        <x:v>0.00682782226716592</x:v>
       </x:c>
       <x:c r="K6" s="29" t="str">
         <x:f>""</x:f>
@@ -2732,11 +2732,11 @@
       </x:c>
       <x:c r="J7" s="29" t="n">
         <x:f>MIN(1,I7/'Assumptions'!$B$9)</x:f>
-        <x:v>0.013212410193757892</x:v>
+        <x:v>0.01320844974682248</x:v>
       </x:c>
       <x:c r="K7" s="29" t="n">
         <x:f>J7-J6</x:f>
-        <x:v>0.006382540659252363</x:v>
+        <x:v>0.006380627479656559</x:v>
       </x:c>
       <x:c r="L7" s="17" t="str">
         <x:f>IF(J7&gt;='Assumptions'!$G$16,"A",IF(J7&gt;='Assumptions'!$G$17,"B",IF(J7&gt;='Assumptions'!$G$18,"C",IF(J7&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2782,11 +2782,11 @@
       </x:c>
       <x:c r="J8" s="29" t="n">
         <x:f>MIN(1,I8/'Assumptions'!$B$9)</x:f>
-        <x:v>0.020077810262916846</x:v>
+        <x:v>0.020071791898291506</x:v>
       </x:c>
       <x:c r="K8" s="29" t="n">
         <x:f>J8-J7</x:f>
-        <x:v>0.0068654000691589535</x:v>
+        <x:v>0.006863342151469026</x:v>
       </x:c>
       <x:c r="L8" s="17" t="str">
         <x:f>IF(J8&gt;='Assumptions'!$G$16,"A",IF(J8&gt;='Assumptions'!$G$17,"B",IF(J8&gt;='Assumptions'!$G$18,"C",IF(J8&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2832,11 +2832,11 @@
       </x:c>
       <x:c r="J9" s="29" t="n">
         <x:f>MIN(1,I9/'Assumptions'!$B$9)</x:f>
-        <x:v>0.028148718558294105</x:v>
+        <x:v>0.02814028092242638</x:v>
       </x:c>
       <x:c r="K9" s="29" t="n">
         <x:f>J9-J8</x:f>
-        <x:v>0.008070908295377259</x:v>
+        <x:v>0.008068489024134873</x:v>
       </x:c>
       <x:c r="L9" s="17" t="str">
         <x:f>IF(J9&gt;='Assumptions'!$G$16,"A",IF(J9&gt;='Assumptions'!$G$17,"B",IF(J9&gt;='Assumptions'!$G$18,"C",IF(J9&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2882,11 +2882,11 @@
       </x:c>
       <x:c r="J10" s="29" t="n">
         <x:f>MIN(1,I10/'Assumptions'!$B$9)</x:f>
-        <x:v>0.0375667289867675</x:v>
+        <x:v>0.037555468283042195</x:v>
       </x:c>
       <x:c r="K10" s="29" t="n">
         <x:f>J10-J9</x:f>
-        <x:v>0.009418010428473397</x:v>
+        <x:v>0.009415187360615817</x:v>
       </x:c>
       <x:c r="L10" s="17" t="str">
         <x:f>IF(J10&gt;='Assumptions'!$G$16,"A",IF(J10&gt;='Assumptions'!$G$17,"B",IF(J10&gt;='Assumptions'!$G$18,"C",IF(J10&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2932,11 +2932,11 @@
       </x:c>
       <x:c r="J11" s="29" t="n">
         <x:f>MIN(1,I11/'Assumptions'!$B$9)</x:f>
-        <x:v>0.06635913961769906</x:v>
+        <x:v>0.06633924833009283</x:v>
       </x:c>
       <x:c r="K11" s="29" t="n">
         <x:f>J11-J10</x:f>
-        <x:v>0.028792410630931554</x:v>
+        <x:v>0.028783780047050636</x:v>
       </x:c>
       <x:c r="L11" s="17" t="str">
         <x:f>IF(J11&gt;='Assumptions'!$G$16,"A",IF(J11&gt;='Assumptions'!$G$17,"B",IF(J11&gt;='Assumptions'!$G$18,"C",IF(J11&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -2982,11 +2982,11 @@
       </x:c>
       <x:c r="J12" s="29" t="n">
         <x:f>MIN(1,I12/'Assumptions'!$B$9)</x:f>
-        <x:v>0.08728779219871709</x:v>
+        <x:v>0.08726162750476324</x:v>
       </x:c>
       <x:c r="K12" s="29" t="n">
         <x:f>J12-J11</x:f>
-        <x:v>0.02092865258101803</x:v>
+        <x:v>0.020922379174670408</x:v>
       </x:c>
       <x:c r="L12" s="17" t="str">
         <x:f>IF(J12&gt;='Assumptions'!$G$16,"A",IF(J12&gt;='Assumptions'!$G$17,"B",IF(J12&gt;='Assumptions'!$G$18,"C",IF(J12&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3032,11 +3032,11 @@
       </x:c>
       <x:c r="J13" s="29" t="n">
         <x:f>MIN(1,I13/'Assumptions'!$B$9)</x:f>
-        <x:v>0.14710906322515388</x:v>
+        <x:v>0.14706496698305438</x:v>
       </x:c>
       <x:c r="K13" s="29" t="n">
         <x:f>J13-J12</x:f>
-        <x:v>0.05982127102643679</x:v>
+        <x:v>0.05980333947829114</x:v>
       </x:c>
       <x:c r="L13" s="17" t="str">
         <x:f>IF(J13&gt;='Assumptions'!$G$16,"A",IF(J13&gt;='Assumptions'!$G$17,"B",IF(J13&gt;='Assumptions'!$G$18,"C",IF(J13&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3082,11 +3082,11 @@
       </x:c>
       <x:c r="J14" s="29" t="n">
         <x:f>MIN(1,I14/'Assumptions'!$B$9)</x:f>
-        <x:v>0.17518649830077868</x:v>
+        <x:v>0.17513398579018094</x:v>
       </x:c>
       <x:c r="K14" s="29" t="n">
         <x:f>J14-J13</x:f>
-        <x:v>0.028077435075624796</x:v>
+        <x:v>0.02806901880712656</x:v>
       </x:c>
       <x:c r="L14" s="17" t="str">
         <x:f>IF(J14&gt;='Assumptions'!$G$16,"A",IF(J14&gt;='Assumptions'!$G$17,"B",IF(J14&gt;='Assumptions'!$G$18,"C",IF(J14&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3132,11 +3132,11 @@
       </x:c>
       <x:c r="J15" s="29" t="n">
         <x:f>MIN(1,I15/'Assumptions'!$B$9)</x:f>
-        <x:v>0.31204191629301636</x:v>
+        <x:v>0.31194838109141576</x:v>
       </x:c>
       <x:c r="K15" s="29" t="n">
         <x:f>J15-J14</x:f>
-        <x:v>0.1368554179922377</x:v>
+        <x:v>0.13681439530123482</x:v>
       </x:c>
       <x:c r="L15" s="17" t="str">
         <x:f>IF(J15&gt;='Assumptions'!$G$16,"A",IF(J15&gt;='Assumptions'!$G$17,"B",IF(J15&gt;='Assumptions'!$G$18,"C",IF(J15&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3182,11 +3182,11 @@
       </x:c>
       <x:c r="J16" s="29" t="n">
         <x:f>MIN(1,I16/'Assumptions'!$B$9)</x:f>
-        <x:v>0.37598995605326785</x:v>
+        <x:v>0.37587725229616675</x:v>
       </x:c>
       <x:c r="K16" s="29" t="n">
         <x:f>J16-J15</x:f>
-        <x:v>0.06394803976025148</x:v>
+        <x:v>0.06392887120475099</x:v>
       </x:c>
       <x:c r="L16" s="17" t="str">
         <x:f>IF(J16&gt;='Assumptions'!$G$16,"A",IF(J16&gt;='Assumptions'!$G$17,"B",IF(J16&gt;='Assumptions'!$G$18,"C",IF(J16&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3232,11 +3232,11 @@
       </x:c>
       <x:c r="J17" s="33" t="n">
         <x:f>MIN(1,I17/'Assumptions'!$B$9)</x:f>
-        <x:v>0.503968053473009</x:v>
+        <x:v>0.5038169880198742</x:v>
       </x:c>
       <x:c r="K17" s="33" t="n">
         <x:f>J17-J16</x:f>
-        <x:v>0.12797809741974114</x:v>
+        <x:v>0.12793973572370743</x:v>
       </x:c>
       <x:c r="L17" s="23" t="str">
         <x:f>IF(J17&gt;='Assumptions'!$G$16,"A",IF(J17&gt;='Assumptions'!$G$17,"B",IF(J17&gt;='Assumptions'!$G$18,"C",IF(J17&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3282,11 +3282,11 @@
       </x:c>
       <x:c r="J18" s="33" t="n">
         <x:f>MIN(1,I18/'Assumptions'!$B$9)</x:f>
-        <x:v>0.6610888725937321</x:v>
+        <x:v>0.660890709854224</x:v>
       </x:c>
       <x:c r="K18" s="33" t="n">
         <x:f>J18-J17</x:f>
-        <x:v>0.15712081912072307</x:v>
+        <x:v>0.15707372183434987</x:v>
       </x:c>
       <x:c r="L18" s="23" t="str">
         <x:f>IF(J18&gt;='Assumptions'!$G$16,"A",IF(J18&gt;='Assumptions'!$G$17,"B",IF(J18&gt;='Assumptions'!$G$18,"C",IF(J18&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3332,11 +3332,11 @@
       </x:c>
       <x:c r="J19" s="33" t="n">
         <x:f>MIN(1,I19/'Assumptions'!$B$9)</x:f>
-        <x:v>0.8486854625531765</x:v>
+        <x:v>0.8484310673527545</x:v>
       </x:c>
       <x:c r="K19" s="33" t="n">
         <x:f>J19-J18</x:f>
-        <x:v>0.1875965899594444</x:v>
+        <x:v>0.18754035749853049</x:v>
       </x:c>
       <x:c r="L19" s="23" t="str">
         <x:f>IF(J19&gt;='Assumptions'!$G$16,"A",IF(J19&gt;='Assumptions'!$G$17,"B",IF(J19&gt;='Assumptions'!$G$18,"C",IF(J19&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3386,7 +3386,7 @@
       </x:c>
       <x:c r="K20" s="33" t="n">
         <x:f>J20-J19</x:f>
-        <x:v>0.15131453744682355</x:v>
+        <x:v>0.15156893264724547</x:v>
       </x:c>
       <x:c r="L20" s="23" t="str">
         <x:f>IF(J20&gt;='Assumptions'!$G$16,"A",IF(J20&gt;='Assumptions'!$G$17,"B",IF(J20&gt;='Assumptions'!$G$18,"C",IF(J20&gt;='Assumptions'!$G$19,"D","F"))))</x:f>
@@ -3654,7 +3654,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R642f4eca3d8d4f6f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3841752e906a4cee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3819,13 +3819,13 @@
         <x:v>U.S. resident population</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
-        <x:v>342697245</x:v>
+        <x:v>342800000</x:v>
       </x:c>
       <x:c r="C7" s="17" t="str">
         <x:v>people</x:v>
       </x:c>
       <x:c r="D7" s="17" t="str">
-        <x:v>Census Population Clock, 2026-07-26</x:v>
+        <x:v>User-specified rounded estimate; Census Population Clock</x:v>
       </x:c>
       <x:c r="F7" s="17" t="str">
         <x:v>Uncached input</x:v>
@@ -3874,7 +3874,7 @@
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f>B7*B8</x:f>
-        <x:v>171348622.5</x:v>
+        <x:v>171400000</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>people</x:v>
@@ -3952,7 +3952,7 @@
       </x:c>
       <x:c r="B12" s="18" t="n">
         <x:f>B9*I11/B24</x:f>
-        <x:v>35969061.89186608</x:v>
+        <x:v>35979846.92445279</x:v>
       </x:c>
       <x:c r="C12" s="17" t="str">
         <x:v>H100e</x:v>
@@ -4275,7 +4275,7 @@
       </x:c>
       <x:c r="B32" s="20" t="n">
         <x:f>INDEX('Quarterly Model'!$C$6:$C$25,B31-1)+(B12-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))/(INDEX('Quarterly Model'!$E$6:$E$25,B31)-INDEX('Quarterly Model'!$E$6:$E$25,B31-1))*(INDEX('Quarterly Model'!$C$6:$C$25,B31)-INDEX('Quarterly Model'!$C$6:$C$25,B31-1))</x:f>
-        <x:v>46631.98192288111</x:v>
+        <x:v>46632.108708204854</x:v>
       </x:c>
       <x:c r="C32" s="17" t="str">
         <x:v>date</x:v>
@@ -4707,7 +4707,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a04d19057f54e02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5252af36a5c0462d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4865,7 +4865,7 @@
         <x:v>Country filter and current site registry</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9" ht="21.600000381469727" hidden="0" customHeight="1">
       <x:c r="A9" s="17" t="str">
         <x:v>SRC-004</x:v>
       </x:c>
@@ -4882,7 +4882,7 @@
         <x:v>https://www.census.gov/popclock/</x:v>
       </x:c>
       <x:c r="F9" s="17" t="str">
-        <x:v>342,697,245 resident population; threshold uses 50%</x:v>
+        <x:v>Model uses the user-specified rounded estimate of 342.8M residents; the selected target is 50%, or 171.4M users</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="32.400001525878906" hidden="0" customHeight="1">
@@ -4932,7 +4932,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R273427cf55b242c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R41270e56dbdd4721"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>